<commit_message>
Fix validation XLSForm settings IDs
</commit_message>
<xml_diff>
--- a/docs/validation/forms/sentinel_validation_central.xlsx
+++ b/docs/validation/forms/sentinel_validation_central.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R66a04e7fbd28488f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R189073635dfa467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R29172858fbdf4722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R91377686b20e4957"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R9baed3db2b7d4a78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R0c1acae659994856"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -472,37 +472,35 @@
   <x:cols>
     <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="7" t="str">
         <x:v>form_title</x:v>
       </x:c>
-      <x:c r="B1" t="str">
+      <x:c r="B1" s="7" t="str">
+        <x:v>form_id</x:v>
+      </x:c>
+      <x:c r="C1" s="7" t="str">
+        <x:v>version</x:v>
+      </x:c>
+      <x:c r="D1" s="7" t="str">
+        <x:v>instance_name</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
         <x:v>Sentinel Central validation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="7" t="str">
-        <x:v>form_id</x:v>
       </x:c>
       <x:c r="B2" t="str">
         <x:v>sentinel_validation_central</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="7" t="str">
-        <x:v>version</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
+      <x:c r="C2" t="str">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="7" t="str">
-        <x:v>instance_name</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
+      <x:c r="D2" t="str">
         <x:v>${validation_run_id}_${test_case_id}</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Fix validation form instance names
</commit_message>
<xml_diff>
--- a/docs/validation/forms/sentinel_validation_central.xlsx
+++ b/docs/validation/forms/sentinel_validation_central.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R91377686b20e4957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R9baed3db2b7d4a78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R0c1acae659994856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Rea736656567f4cdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Ra53487d2e6a14c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R18bfea04d8504a89"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -501,7 +501,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>${validation_run_id}_${test_case_id}</x:v>
+        <x:v>concat(${validation_run_id}, '_', ${test_case_id})</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>